<commit_message>
Support Pulse refresh 2026-06-10
</commit_message>
<xml_diff>
--- a/support-pulse/support_pulse.xlsx
+++ b/support-pulse/support_pulse.xlsx
@@ -5903,7 +5903,7 @@
         <v>3</v>
       </c>
       <c r="S89" t="n">
-        <v>0.9</v>
+        <v>1.4</v>
       </c>
     </row>
     <row r="90">
@@ -5929,10 +5929,10 @@
         <v>41</v>
       </c>
       <c r="F90" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="G90" t="n">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="I90" t="n">
         <v>5</v>
@@ -5956,16 +5956,16 @@
         <v>6</v>
       </c>
       <c r="P90" t="n">
-        <v>70</v>
+        <v>71</v>
       </c>
       <c r="Q90" t="n">
         <v>0</v>
       </c>
       <c r="R90" t="n">
-        <v>29.4</v>
+        <v>28.7</v>
       </c>
       <c r="S90" t="n">
-        <v>1.1</v>
+        <v>2.2</v>
       </c>
     </row>
     <row r="91">
@@ -5988,13 +5988,13 @@
         <v>0</v>
       </c>
       <c r="E91" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="F91" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="G91" t="n">
-        <v>0</v>
+        <v>6</v>
       </c>
       <c r="I91" t="n">
         <v>0</v>
@@ -6018,10 +6018,16 @@
         <v>1</v>
       </c>
       <c r="P91" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="Q91" t="n">
         <v>0</v>
+      </c>
+      <c r="R91" t="n">
+        <v>8.5</v>
+      </c>
+      <c r="S91" t="n">
+        <v>0.2</v>
       </c>
     </row>
   </sheetData>
@@ -6983,13 +6989,13 @@
         <v>4</v>
       </c>
       <c r="E15" t="n">
-        <v>66</v>
+        <v>69</v>
       </c>
       <c r="F15" t="n">
-        <v>36</v>
+        <v>40</v>
       </c>
       <c r="G15" t="n">
-        <v>106</v>
+        <v>113</v>
       </c>
       <c r="I15" t="n">
         <v>6</v>
@@ -7013,16 +7019,16 @@
         <v>9</v>
       </c>
       <c r="P15" t="n">
-        <v>115</v>
+        <v>122</v>
       </c>
       <c r="Q15" t="n">
         <v>0</v>
       </c>
       <c r="R15" t="n">
-        <v>18.9</v>
+        <v>17.7</v>
       </c>
       <c r="S15" t="n">
-        <v>1</v>
+        <v>1.9</v>
       </c>
     </row>
   </sheetData>
@@ -7364,13 +7370,13 @@
         <v>24</v>
       </c>
       <c r="E5" t="n">
-        <v>137</v>
+        <v>140</v>
       </c>
       <c r="F5" t="n">
-        <v>121</v>
+        <v>125</v>
       </c>
       <c r="G5" t="n">
-        <v>282</v>
+        <v>289</v>
       </c>
       <c r="I5" t="n">
         <v>13</v>
@@ -7394,7 +7400,7 @@
         <v>31</v>
       </c>
       <c r="P5" t="n">
-        <v>313</v>
+        <v>320</v>
       </c>
       <c r="Q5" t="n">
         <v>12.9</v>
@@ -7403,7 +7409,7 @@
         <v>10.1</v>
       </c>
       <c r="S5" t="n">
-        <v>3.4</v>
+        <v>3.6</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Support Pulse: add Volume-by-type tab (main + sub categories)
- Categorize Intercom conversations into main→sub taxonomy (CATEGORY_RULES in refresh_volume.py)
- New long-format support_categories_daily.csv (per day×main×sub), upserted like daily
- Dashboard 'By type' tab: stacked-area category trend + stacked-bar totals + main/sub breakdown table
- All respect the granularity toggle and From/To date pickers

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/support-pulse/support_pulse.xlsx
+++ b/support-pulse/support_pulse.xlsx
@@ -628,13 +628,13 @@
         <v>0</v>
       </c>
       <c r="E3" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F3" t="n">
-        <v>7</v>
+        <v>0</v>
       </c>
       <c r="G3" t="n">
-        <v>8</v>
+        <v>0</v>
       </c>
       <c r="I3" t="n">
         <v>3</v>
@@ -658,16 +658,10 @@
         <v>4</v>
       </c>
       <c r="P3" t="n">
-        <v>12</v>
+        <v>4</v>
       </c>
       <c r="Q3" t="n">
         <v>0</v>
-      </c>
-      <c r="R3" t="n">
-        <v>5.7</v>
-      </c>
-      <c r="S3" t="n">
-        <v>36.6</v>
       </c>
     </row>
     <row r="4">
@@ -2432,7 +2426,7 @@
         <v>966.2</v>
       </c>
       <c r="S32" t="n">
-        <v>8.1</v>
+        <v>22.3</v>
       </c>
     </row>
     <row r="33">
@@ -2839,7 +2833,7 @@
         <v>0</v>
       </c>
       <c r="K39" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="L39" t="n">
         <v>1</v>
@@ -5177,7 +5171,7 @@
         <v>34.7</v>
       </c>
       <c r="S77" t="n">
-        <v>3.9</v>
+        <v>17.4</v>
       </c>
     </row>
     <row r="78">
@@ -5324,13 +5318,13 @@
         <v>0</v>
       </c>
       <c r="E80" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F80" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="G80" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="I80" t="n">
         <v>1</v>
@@ -5354,10 +5348,16 @@
         <v>1</v>
       </c>
       <c r="P80" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="Q80" t="n">
         <v>0</v>
+      </c>
+      <c r="R80" t="n">
+        <v>114</v>
+      </c>
+      <c r="S80" t="n">
+        <v>11</v>
       </c>
     </row>
     <row r="81">
@@ -5534,7 +5534,7 @@
         <v>33.3</v>
       </c>
       <c r="R83" t="n">
-        <v>3.2</v>
+        <v>176.8</v>
       </c>
       <c r="S83" t="n">
         <v>3.9</v>
@@ -5661,7 +5661,7 @@
         <v>6.8</v>
       </c>
       <c r="S85" t="n">
-        <v>5.3</v>
+        <v>6.9</v>
       </c>
     </row>
     <row r="86">
@@ -5720,7 +5720,7 @@
         <v>14.3</v>
       </c>
       <c r="R86" t="n">
-        <v>2.1</v>
+        <v>171.3</v>
       </c>
       <c r="S86" t="n">
         <v>2.6</v>
@@ -5841,7 +5841,7 @@
         <v>0</v>
       </c>
       <c r="S88" t="n">
-        <v>8</v>
+        <v>9.9</v>
       </c>
     </row>
     <row r="89">
@@ -5903,7 +5903,7 @@
         <v>3</v>
       </c>
       <c r="S89" t="n">
-        <v>1.4</v>
+        <v>1.8</v>
       </c>
     </row>
     <row r="90">
@@ -5962,10 +5962,10 @@
         <v>0</v>
       </c>
       <c r="R90" t="n">
-        <v>28.7</v>
+        <v>35.8</v>
       </c>
       <c r="S90" t="n">
-        <v>2.2</v>
+        <v>2.6</v>
       </c>
     </row>
     <row r="91">
@@ -5985,28 +5985,28 @@
         </is>
       </c>
       <c r="D91" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="E91" t="n">
+        <v>21</v>
+      </c>
+      <c r="F91" t="n">
+        <v>19</v>
+      </c>
+      <c r="G91" t="n">
+        <v>44</v>
+      </c>
+      <c r="I91" t="n">
+        <v>6</v>
+      </c>
+      <c r="J91" t="n">
+        <v>0</v>
+      </c>
+      <c r="K91" t="n">
         <v>3</v>
       </c>
-      <c r="F91" t="n">
-        <v>3</v>
-      </c>
-      <c r="G91" t="n">
-        <v>6</v>
-      </c>
-      <c r="I91" t="n">
-        <v>0</v>
-      </c>
-      <c r="J91" t="n">
-        <v>0</v>
-      </c>
-      <c r="K91" t="n">
-        <v>0</v>
-      </c>
       <c r="L91" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="M91" t="n">
         <v>0</v>
@@ -6015,19 +6015,19 @@
         <v>0</v>
       </c>
       <c r="O91" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="P91" t="n">
-        <v>7</v>
+        <v>52</v>
       </c>
       <c r="Q91" t="n">
         <v>0</v>
       </c>
       <c r="R91" t="n">
-        <v>8.5</v>
+        <v>4.6</v>
       </c>
       <c r="S91" t="n">
-        <v>0.2</v>
+        <v>0.6</v>
       </c>
     </row>
   </sheetData>
@@ -6183,13 +6183,13 @@
         <v>0</v>
       </c>
       <c r="E2" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="F2" t="n">
-        <v>16</v>
+        <v>9</v>
       </c>
       <c r="G2" t="n">
-        <v>17</v>
+        <v>9</v>
       </c>
       <c r="I2" t="n">
         <v>4</v>
@@ -6213,16 +6213,16 @@
         <v>7</v>
       </c>
       <c r="P2" t="n">
-        <v>24</v>
+        <v>16</v>
       </c>
       <c r="Q2" t="n">
         <v>14.3</v>
       </c>
       <c r="R2" t="n">
-        <v>3.2</v>
+        <v>1.3</v>
       </c>
       <c r="S2" t="n">
-        <v>24.4</v>
+        <v>13.6</v>
       </c>
     </row>
     <row r="3">
@@ -6470,7 +6470,7 @@
         <v>275.7</v>
       </c>
       <c r="S6" t="n">
-        <v>28.4</v>
+        <v>32.4</v>
       </c>
     </row>
     <row r="7">
@@ -6508,7 +6508,7 @@
         <v>0</v>
       </c>
       <c r="K7" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L7" t="n">
         <v>10</v>
@@ -6865,13 +6865,13 @@
         <v>15</v>
       </c>
       <c r="E13" t="n">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="F13" t="n">
-        <v>76</v>
+        <v>80</v>
       </c>
       <c r="G13" t="n">
-        <v>116</v>
+        <v>121</v>
       </c>
       <c r="I13" t="n">
         <v>32</v>
@@ -6895,16 +6895,16 @@
         <v>48</v>
       </c>
       <c r="P13" t="n">
-        <v>164</v>
+        <v>169</v>
       </c>
       <c r="Q13" t="n">
         <v>14.6</v>
       </c>
       <c r="R13" t="n">
-        <v>11</v>
+        <v>13.9</v>
       </c>
       <c r="S13" t="n">
-        <v>6.6</v>
+        <v>9.1</v>
       </c>
     </row>
     <row r="14">
@@ -6963,10 +6963,10 @@
         <v>18.2</v>
       </c>
       <c r="R14" t="n">
-        <v>5.6</v>
+        <v>71.7</v>
       </c>
       <c r="S14" t="n">
-        <v>4.6</v>
+        <v>4.9</v>
       </c>
     </row>
     <row r="15">
@@ -6986,28 +6986,28 @@
         </is>
       </c>
       <c r="D15" t="n">
+        <v>8</v>
+      </c>
+      <c r="E15" t="n">
+        <v>87</v>
+      </c>
+      <c r="F15" t="n">
+        <v>56</v>
+      </c>
+      <c r="G15" t="n">
+        <v>151</v>
+      </c>
+      <c r="I15" t="n">
+        <v>12</v>
+      </c>
+      <c r="J15" t="n">
+        <v>0</v>
+      </c>
+      <c r="K15" t="n">
         <v>4</v>
       </c>
-      <c r="E15" t="n">
-        <v>69</v>
-      </c>
-      <c r="F15" t="n">
-        <v>40</v>
-      </c>
-      <c r="G15" t="n">
-        <v>113</v>
-      </c>
-      <c r="I15" t="n">
-        <v>6</v>
-      </c>
-      <c r="J15" t="n">
-        <v>0</v>
-      </c>
-      <c r="K15" t="n">
-        <v>1</v>
-      </c>
       <c r="L15" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="M15" t="n">
         <v>0</v>
@@ -7016,16 +7016,16 @@
         <v>0</v>
       </c>
       <c r="O15" t="n">
-        <v>9</v>
+        <v>16</v>
       </c>
       <c r="P15" t="n">
-        <v>122</v>
+        <v>167</v>
       </c>
       <c r="Q15" t="n">
         <v>0</v>
       </c>
       <c r="R15" t="n">
-        <v>17.7</v>
+        <v>17</v>
       </c>
       <c r="S15" t="n">
         <v>1.9</v>
@@ -7184,13 +7184,13 @@
         <v>0</v>
       </c>
       <c r="E2" t="n">
-        <v>23</v>
+        <v>22</v>
       </c>
       <c r="F2" t="n">
-        <v>161</v>
+        <v>154</v>
       </c>
       <c r="G2" t="n">
-        <v>184</v>
+        <v>176</v>
       </c>
       <c r="I2" t="n">
         <v>19</v>
@@ -7214,16 +7214,16 @@
         <v>40</v>
       </c>
       <c r="P2" t="n">
-        <v>224</v>
+        <v>216</v>
       </c>
       <c r="Q2" t="n">
         <v>17.5</v>
       </c>
       <c r="R2" t="n">
+        <v>34.5</v>
+      </c>
+      <c r="S2" t="n">
         <v>33.1</v>
-      </c>
-      <c r="S2" t="n">
-        <v>33.3</v>
       </c>
     </row>
     <row r="3">
@@ -7261,7 +7261,7 @@
         <v>1</v>
       </c>
       <c r="K3" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L3" t="n">
         <v>58</v>
@@ -7285,7 +7285,7 @@
         <v>117.2</v>
       </c>
       <c r="S3" t="n">
-        <v>40.5</v>
+        <v>41.6</v>
       </c>
     </row>
     <row r="4">
@@ -7308,13 +7308,13 @@
         <v>15</v>
       </c>
       <c r="E4" t="n">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="F4" t="n">
-        <v>374</v>
+        <v>378</v>
       </c>
       <c r="G4" t="n">
-        <v>473</v>
+        <v>478</v>
       </c>
       <c r="I4" t="n">
         <v>68</v>
@@ -7338,16 +7338,16 @@
         <v>128</v>
       </c>
       <c r="P4" t="n">
-        <v>601</v>
+        <v>606</v>
       </c>
       <c r="Q4" t="n">
         <v>14.1</v>
       </c>
       <c r="R4" t="n">
-        <v>61.8</v>
+        <v>62.1</v>
       </c>
       <c r="S4" t="n">
-        <v>18.6</v>
+        <v>19</v>
       </c>
     </row>
     <row r="5">
@@ -7367,28 +7367,28 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="E5" t="n">
-        <v>140</v>
+        <v>158</v>
       </c>
       <c r="F5" t="n">
-        <v>125</v>
+        <v>141</v>
       </c>
       <c r="G5" t="n">
-        <v>289</v>
+        <v>327</v>
       </c>
       <c r="I5" t="n">
-        <v>13</v>
+        <v>19</v>
       </c>
       <c r="J5" t="n">
         <v>0</v>
       </c>
       <c r="K5" t="n">
-        <v>1</v>
+        <v>4</v>
       </c>
       <c r="L5" t="n">
-        <v>18</v>
+        <v>19</v>
       </c>
       <c r="M5" t="n">
         <v>0</v>
@@ -7397,16 +7397,16 @@
         <v>0</v>
       </c>
       <c r="O5" t="n">
-        <v>31</v>
+        <v>38</v>
       </c>
       <c r="P5" t="n">
-        <v>320</v>
+        <v>365</v>
       </c>
       <c r="Q5" t="n">
-        <v>12.9</v>
+        <v>10.5</v>
       </c>
       <c r="R5" t="n">
-        <v>10.1</v>
+        <v>47.6</v>
       </c>
       <c r="S5" t="n">
         <v>3.6</v>

</xml_diff>

<commit_message>
Support Pulse: add 'By user type' tab + sharpen categorization
- Classify each conversation to a primary user persona (Driver/Dispatcher/Biller/
  Reporting/Admin/...) from request content + the contact's Intercom Roles attribute
- New support_usertypes_daily.csv (long format), upserted like categories
- 'By user type' tab: persona trend (stacked area) + totals bar + breakdown table; respects date pickers
- Categorize now also reads conversation subject/body text, not just tags —
  Uncategorized dropped ~24% -> ~5%
- Contact-roles cache kept local + gitignored (never published); no customer names anywhere

Co-Authored-By: Claude Opus 4.8 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/support-pulse/support_pulse.xlsx
+++ b/support-pulse/support_pulse.xlsx
@@ -431,7 +431,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S91"/>
+  <dimension ref="A1:S93"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14" customWidth="1" min="1" max="1"/>
@@ -5965,7 +5965,7 @@
         <v>35.8</v>
       </c>
       <c r="S90" t="n">
-        <v>2.6</v>
+        <v>3.7</v>
       </c>
     </row>
     <row r="91">
@@ -5985,19 +5985,19 @@
         </is>
       </c>
       <c r="D91" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="E91" t="n">
-        <v>21</v>
+        <v>24</v>
       </c>
       <c r="F91" t="n">
-        <v>19</v>
+        <v>25</v>
       </c>
       <c r="G91" t="n">
-        <v>44</v>
+        <v>55</v>
       </c>
       <c r="I91" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="J91" t="n">
         <v>0</v>
@@ -6015,19 +6015,137 @@
         <v>0</v>
       </c>
       <c r="O91" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="P91" t="n">
-        <v>52</v>
+        <v>64</v>
       </c>
       <c r="Q91" t="n">
         <v>0</v>
       </c>
       <c r="R91" t="n">
-        <v>4.6</v>
+        <v>20.7</v>
       </c>
       <c r="S91" t="n">
-        <v>0.6</v>
+        <v>2.4</v>
+      </c>
+    </row>
+    <row r="92">
+      <c r="A92" t="inlineStr">
+        <is>
+          <t>2026-06-11</t>
+        </is>
+      </c>
+      <c r="B92" t="inlineStr">
+        <is>
+          <t>2026-06-11</t>
+        </is>
+      </c>
+      <c r="C92" t="inlineStr">
+        <is>
+          <t>2026-06-11</t>
+        </is>
+      </c>
+      <c r="D92" t="n">
+        <v>2</v>
+      </c>
+      <c r="E92" t="n">
+        <v>10</v>
+      </c>
+      <c r="F92" t="n">
+        <v>11</v>
+      </c>
+      <c r="G92" t="n">
+        <v>23</v>
+      </c>
+      <c r="I92" t="n">
+        <v>1</v>
+      </c>
+      <c r="J92" t="n">
+        <v>0</v>
+      </c>
+      <c r="K92" t="n">
+        <v>0</v>
+      </c>
+      <c r="L92" t="n">
+        <v>3</v>
+      </c>
+      <c r="M92" t="n">
+        <v>0</v>
+      </c>
+      <c r="N92" t="n">
+        <v>0</v>
+      </c>
+      <c r="O92" t="n">
+        <v>4</v>
+      </c>
+      <c r="P92" t="n">
+        <v>27</v>
+      </c>
+      <c r="Q92" t="n">
+        <v>0</v>
+      </c>
+      <c r="R92" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="S92" t="n">
+        <v>0.8</v>
+      </c>
+    </row>
+    <row r="93">
+      <c r="A93" t="inlineStr">
+        <is>
+          <t>2026-06-12</t>
+        </is>
+      </c>
+      <c r="B93" t="inlineStr">
+        <is>
+          <t>2026-06-12</t>
+        </is>
+      </c>
+      <c r="C93" t="inlineStr">
+        <is>
+          <t>2026-06-12</t>
+        </is>
+      </c>
+      <c r="D93" t="n">
+        <v>0</v>
+      </c>
+      <c r="E93" t="n">
+        <v>0</v>
+      </c>
+      <c r="F93" t="n">
+        <v>0</v>
+      </c>
+      <c r="G93" t="n">
+        <v>0</v>
+      </c>
+      <c r="I93" t="n">
+        <v>0</v>
+      </c>
+      <c r="J93" t="n">
+        <v>0</v>
+      </c>
+      <c r="K93" t="n">
+        <v>0</v>
+      </c>
+      <c r="L93" t="n">
+        <v>2</v>
+      </c>
+      <c r="M93" t="n">
+        <v>0</v>
+      </c>
+      <c r="N93" t="n">
+        <v>0</v>
+      </c>
+      <c r="O93" t="n">
+        <v>2</v>
+      </c>
+      <c r="P93" t="n">
+        <v>2</v>
+      </c>
+      <c r="Q93" t="n">
+        <v>0</v>
       </c>
     </row>
   </sheetData>
@@ -6986,19 +7104,19 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="E15" t="n">
-        <v>87</v>
+        <v>100</v>
       </c>
       <c r="F15" t="n">
-        <v>56</v>
+        <v>73</v>
       </c>
       <c r="G15" t="n">
-        <v>151</v>
+        <v>185</v>
       </c>
       <c r="I15" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="J15" t="n">
         <v>0</v>
@@ -7007,7 +7125,7 @@
         <v>4</v>
       </c>
       <c r="L15" t="n">
-        <v>4</v>
+        <v>9</v>
       </c>
       <c r="M15" t="n">
         <v>0</v>
@@ -7016,19 +7134,19 @@
         <v>0</v>
       </c>
       <c r="O15" t="n">
-        <v>16</v>
+        <v>23</v>
       </c>
       <c r="P15" t="n">
-        <v>167</v>
+        <v>208</v>
       </c>
       <c r="Q15" t="n">
         <v>0</v>
       </c>
       <c r="R15" t="n">
-        <v>17</v>
+        <v>19.4</v>
       </c>
       <c r="S15" t="n">
-        <v>1.9</v>
+        <v>2.6</v>
       </c>
     </row>
   </sheetData>
@@ -7367,19 +7485,19 @@
         </is>
       </c>
       <c r="D5" t="n">
-        <v>28</v>
+        <v>32</v>
       </c>
       <c r="E5" t="n">
+        <v>171</v>
+      </c>
+      <c r="F5" t="n">
         <v>158</v>
       </c>
-      <c r="F5" t="n">
-        <v>141</v>
-      </c>
       <c r="G5" t="n">
-        <v>327</v>
+        <v>361</v>
       </c>
       <c r="I5" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="J5" t="n">
         <v>0</v>
@@ -7388,7 +7506,7 @@
         <v>4</v>
       </c>
       <c r="L5" t="n">
-        <v>19</v>
+        <v>24</v>
       </c>
       <c r="M5" t="n">
         <v>0</v>
@@ -7397,19 +7515,19 @@
         <v>0</v>
       </c>
       <c r="O5" t="n">
-        <v>38</v>
+        <v>45</v>
       </c>
       <c r="P5" t="n">
-        <v>365</v>
+        <v>406</v>
       </c>
       <c r="Q5" t="n">
-        <v>10.5</v>
+        <v>8.9</v>
       </c>
       <c r="R5" t="n">
-        <v>47.6</v>
+        <v>45.7</v>
       </c>
       <c r="S5" t="n">
-        <v>3.6</v>
+        <v>3.8</v>
       </c>
     </row>
   </sheetData>

</xml_diff>